<commit_message>
Adicionei a logica de edição de contrato no file EditarContrato.js
</commit_message>
<xml_diff>
--- a/db/FARE26RC.xlsx
+++ b/db/FARE26RC.xlsx
@@ -1,29 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Roque Savioli\Desktop\arquivo-projeto\aryoleofar\db\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4DEE0438-0750-4C43-9B65-9796C1798890}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940"/>
   </bookViews>
   <sheets>
-    <sheet name="FARE26RC" sheetId="1" r:id="rId1"/>
+    <sheet sheetId="1" name="FARE26RC" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Database">FARE26RC!$A$1:$N$16</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="64">
   <si>
     <t>DATA</t>
   </si>
@@ -79,6 +73,9 @@
     <t>COOPERTRADICAO CLEVE</t>
   </si>
   <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
     <t>002</t>
   </si>
   <si>
@@ -208,331 +205,34 @@
     <t>20451</t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
+    <t/>
+  </si>
+  <si>
+    <t>teste</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.79998168889431442"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.59999389629810485"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.39997558519241921"/>
-        <bgColor indexed="65"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="10">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -540,157 +240,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="thick">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.39997558519241921"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="42">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="17" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -698,49 +250,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="42">
-    <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
-    <cellStyle name="20% - Ênfase2" xfId="23" builtinId="34" customBuiltin="1"/>
-    <cellStyle name="20% - Ênfase3" xfId="27" builtinId="38" customBuiltin="1"/>
-    <cellStyle name="20% - Ênfase4" xfId="31" builtinId="42" customBuiltin="1"/>
-    <cellStyle name="20% - Ênfase5" xfId="35" builtinId="46" customBuiltin="1"/>
-    <cellStyle name="20% - Ênfase6" xfId="39" builtinId="50" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase1" xfId="20" builtinId="31" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase2" xfId="24" builtinId="35" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase3" xfId="28" builtinId="39" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase4" xfId="32" builtinId="43" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase5" xfId="36" builtinId="47" customBuiltin="1"/>
-    <cellStyle name="40% - Ênfase6" xfId="40" builtinId="51" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase1" xfId="21" builtinId="32" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase2" xfId="25" builtinId="36" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase3" xfId="29" builtinId="40" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase4" xfId="33" builtinId="44" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase5" xfId="37" builtinId="48" customBuiltin="1"/>
-    <cellStyle name="60% - Ênfase6" xfId="41" builtinId="52" customBuiltin="1"/>
-    <cellStyle name="Bom" xfId="6" builtinId="26" customBuiltin="1"/>
-    <cellStyle name="Cálculo" xfId="11" builtinId="22" customBuiltin="1"/>
-    <cellStyle name="Célula de Verificação" xfId="13" builtinId="23" customBuiltin="1"/>
-    <cellStyle name="Célula Vinculada" xfId="12" builtinId="24" customBuiltin="1"/>
-    <cellStyle name="Ênfase1" xfId="18" builtinId="29" customBuiltin="1"/>
-    <cellStyle name="Ênfase2" xfId="22" builtinId="33" customBuiltin="1"/>
-    <cellStyle name="Ênfase3" xfId="26" builtinId="37" customBuiltin="1"/>
-    <cellStyle name="Ênfase4" xfId="30" builtinId="41" customBuiltin="1"/>
-    <cellStyle name="Ênfase5" xfId="34" builtinId="45" customBuiltin="1"/>
-    <cellStyle name="Ênfase6" xfId="38" builtinId="49" customBuiltin="1"/>
-    <cellStyle name="Entrada" xfId="9" builtinId="20" customBuiltin="1"/>
-    <cellStyle name="Neutro" xfId="8" builtinId="28" customBuiltin="1"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Nota" xfId="15" builtinId="10" customBuiltin="1"/>
-    <cellStyle name="Ruim" xfId="7" builtinId="27" customBuiltin="1"/>
-    <cellStyle name="Saída" xfId="10" builtinId="21" customBuiltin="1"/>
-    <cellStyle name="Texto de Aviso" xfId="14" builtinId="11" customBuiltin="1"/>
-    <cellStyle name="Texto Explicativo" xfId="16" builtinId="53" customBuiltin="1"/>
-    <cellStyle name="Título" xfId="1" builtinId="15" customBuiltin="1"/>
-    <cellStyle name="Título 1" xfId="2" builtinId="16" customBuiltin="1"/>
-    <cellStyle name="Título 2" xfId="3" builtinId="17" customBuiltin="1"/>
-    <cellStyle name="Título 3" xfId="4" builtinId="18" customBuiltin="1"/>
-    <cellStyle name="Título 4" xfId="5" builtinId="19" customBuiltin="1"/>
-    <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1052,8 +563,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O16"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O17"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="8.77734375" customWidth="1"/>
     <col min="2" max="2" width="7.77734375" style="1" customWidth="1"/>
@@ -1068,7 +579,7 @@
     <col min="14" max="14" width="14.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1112,7 +623,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>46078</v>
       </c>
@@ -1129,10 +640,10 @@
         <v>17</v>
       </c>
       <c r="O2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>46080</v>
       </c>
@@ -1140,16 +651,16 @@
         <v>14</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G3" s="2">
-        <v>17697.830000000002</v>
+        <v>17697.83</v>
       </c>
       <c r="H3" s="2">
         <v>17432.36</v>
@@ -1158,13 +669,13 @@
         <v>0</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M3" s="3">
         <v>46195</v>
@@ -1173,7 +684,7 @@
         <v>8769.01</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>46080</v>
       </c>
@@ -1181,31 +692,31 @@
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G4" s="2">
-        <v>8795.2199999999993</v>
+        <v>8795.22</v>
       </c>
       <c r="H4" s="2">
-        <v>8663.2900000000009</v>
+        <v>8663.29</v>
       </c>
       <c r="I4" s="2">
         <v>0</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M4" s="3">
         <v>46113</v>
@@ -1214,7 +725,7 @@
         <v>4520.72</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>46098</v>
       </c>
@@ -1222,16 +733,16 @@
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G5" s="2">
-        <v>69953.600000000006</v>
+        <v>69953.6</v>
       </c>
       <c r="H5" s="2">
         <v>68904.3</v>
@@ -1240,22 +751,22 @@
         <v>0</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M5" s="3">
         <v>46213</v>
       </c>
       <c r="N5" s="2">
-        <v>34660.980000000003</v>
-      </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+        <v>34660.98</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>46098</v>
       </c>
@@ -1263,40 +774,40 @@
         <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2">
         <v>72414</v>
       </c>
       <c r="H6" s="2">
-        <v>71327.789999999994</v>
+        <v>71327.79</v>
       </c>
       <c r="I6" s="2">
         <v>0</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M6" s="3">
         <v>46274</v>
       </c>
       <c r="N6" s="2">
-        <v>35762.769999999997</v>
-      </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+        <v>35762.77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>46119</v>
       </c>
@@ -1304,40 +815,40 @@
         <v>14</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G7" s="2">
         <v>35112.78</v>
       </c>
       <c r="H7" s="2">
-        <v>34586.089999999997</v>
+        <v>34586.09</v>
       </c>
       <c r="I7" s="2">
         <v>0</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M7" s="3">
         <v>46286</v>
       </c>
       <c r="N7" s="2">
-        <v>17340.990000000002</v>
-      </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+        <v>17340.99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>46128</v>
       </c>
@@ -1345,13 +856,13 @@
         <v>14</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2">
         <v>18200</v>
@@ -1363,13 +874,13 @@
         <v>0</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M8" s="3">
         <v>46185</v>
@@ -1378,7 +889,7 @@
         <v>9017.83</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>46140</v>
       </c>
@@ -1386,13 +897,13 @@
         <v>14</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G9" s="2">
         <v>70085.16</v>
@@ -1404,22 +915,22 @@
         <v>0</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M9" s="3">
         <v>46266</v>
       </c>
       <c r="N9" s="2">
-        <v>34612.639999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+        <v>34612.64</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>46149</v>
       </c>
@@ -1427,31 +938,31 @@
         <v>14</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G10" s="2">
         <v>42886.66</v>
       </c>
       <c r="H10" s="2">
-        <v>42243.360000000001</v>
+        <v>42243.36</v>
       </c>
       <c r="I10" s="2">
         <v>0</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M10" s="3">
         <v>46227</v>
@@ -1460,7 +971,7 @@
         <v>21428.34</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>46185</v>
       </c>
@@ -1468,13 +979,13 @@
         <v>14</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="G11" s="2">
         <v>70000</v>
@@ -1486,13 +997,13 @@
         <v>0</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M11" s="3">
         <v>46274</v>
@@ -1501,7 +1012,7 @@
         <v>34570.58</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>46205</v>
       </c>
@@ -1509,13 +1020,13 @@
         <v>14</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G12" s="2">
         <v>8738.01</v>
@@ -1527,22 +1038,22 @@
         <v>0</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M12" s="3">
         <v>46266</v>
       </c>
       <c r="N12" s="2">
-        <v>4315.3999999999996</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+        <v>4315.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>46210</v>
       </c>
@@ -1550,16 +1061,16 @@
         <v>14</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G13" s="2">
-        <v>8837.9599999999991</v>
+        <v>8837.96</v>
       </c>
       <c r="H13" s="2">
         <v>8705.39</v>
@@ -1568,13 +1079,13 @@
         <v>0</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M13" s="3">
         <v>46266</v>
@@ -1583,7 +1094,7 @@
         <v>4364.76</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>46248</v>
       </c>
@@ -1591,16 +1102,16 @@
         <v>14</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>46140</v>
       </c>
@@ -1608,16 +1119,16 @@
         <v>14</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G15" s="2">
-        <v>64883.519999999997</v>
+        <v>64883.52</v>
       </c>
       <c r="H15" s="2">
         <v>63910.27</v>
@@ -1626,13 +1137,13 @@
         <v>0</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M15" s="3">
         <v>46296</v>
@@ -1641,7 +1152,7 @@
         <v>32043.73</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>46119</v>
       </c>
@@ -1649,13 +1160,13 @@
         <v>14</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>16</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G16" s="2">
         <v>9326.49</v>
@@ -1667,13 +1178,13 @@
         <v>0</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="M16" s="3">
         <v>46286</v>
@@ -1682,7 +1193,48 @@
         <v>4606.03</v>
       </c>
     </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A17" s="3">
+        <v>46078</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="J17" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="L17" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="M17" t="s">
+        <v>62</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.787401575" bottom="0.787401575" header="0.31496062" footer="0.31496062"/>
 </worksheet>
 </file>
</xml_diff>